<commit_message>
Update final synthetic examples and instructions
</commit_message>
<xml_diff>
--- a/example/synthetic_thickness.xlsx
+++ b/example/synthetic_thickness.xlsx
@@ -22,10 +22,10 @@
     <t>Y</t>
   </si>
   <si>
-    <t>Ketebalan LIM</t>
+    <t>Limonite Thickness</t>
   </si>
   <si>
-    <t>Ketebalan SAP</t>
+    <t>Saprolite Thickness</t>
   </si>
 </sst>
 </file>

</xml_diff>